<commit_message>
Update bitcoin_buys.xlsx after running on 2026-03-08
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D72"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1556,6 +1556,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>0.0007333900000000004</v>
+      </c>
+      <c r="C73" t="n">
+        <v>67494.78449392543</v>
+      </c>
+      <c r="D73" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-03-15
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D73"/>
+  <dimension ref="A1:D74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1572,6 +1572,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>03/15/2026</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>0.0006876999999999994</v>
+      </c>
+      <c r="C74" t="n">
+        <v>71979.06063690569</v>
+      </c>
+      <c r="D74" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-03-22
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1588,6 +1588,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>03/22/2026</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>0.0007122099999999978</v>
+      </c>
+      <c r="C75" t="n">
+        <v>69501.97273276161</v>
+      </c>
+      <c r="D75" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-03-29
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D75"/>
+  <dimension ref="A1:D76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1604,6 +1604,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>03/29/2026</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>0.0007395499999999985</v>
+      </c>
+      <c r="C76" t="n">
+        <v>66932.59414508835</v>
+      </c>
+      <c r="D76" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-04-12
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D76"/>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1620,6 +1620,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>04/12/2026</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>0.0006872399999999987</v>
+      </c>
+      <c r="C77" t="n">
+        <v>72027.23939235216</v>
+      </c>
+      <c r="D77" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-04-19
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D77"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1636,6 +1636,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>04/19/2026</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>0.0006509999999999988</v>
+      </c>
+      <c r="C78" t="n">
+        <v>76036.86635944714</v>
+      </c>
+      <c r="D78" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-04-26
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D78"/>
+  <dimension ref="A1:D79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1652,6 +1652,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>04/26/2026</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>0.0006311600000000056</v>
+      </c>
+      <c r="C79" t="n">
+        <v>78427.02325876095</v>
+      </c>
+      <c r="D79" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-05-03
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D79"/>
+  <dimension ref="A1:D80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1668,6 +1668,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>05/03/2026</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>0.00062976</v>
+      </c>
+      <c r="C80" t="n">
+        <v>78601.37195121951</v>
+      </c>
+      <c r="D80" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-05-10
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D80"/>
+  <dimension ref="A1:D81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1684,6 +1684,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>0.0006100100000000011</v>
+      </c>
+      <c r="C81" t="n">
+        <v>81146.21071785694</v>
+      </c>
+      <c r="D81" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-05-17
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D81"/>
+  <dimension ref="A1:D82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1700,6 +1700,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>05/17/2026</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>0.0006301299999999996</v>
+      </c>
+      <c r="C82" t="n">
+        <v>78555.21876438201</v>
+      </c>
+      <c r="D82" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-05-24
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D82"/>
+  <dimension ref="A1:D83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1716,6 +1716,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>05/24/2026</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>0.0006431299999999987</v>
+      </c>
+      <c r="C83" t="n">
+        <v>76967.33164368029</v>
+      </c>
+      <c r="D83" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-05-31
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D83"/>
+  <dimension ref="A1:D84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1732,6 +1732,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>05/31/2026</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>0.0006656199999999987</v>
+      </c>
+      <c r="C84" t="n">
+        <v>74366.75580661654</v>
+      </c>
+      <c r="D84" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-06-07
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D84"/>
+  <dimension ref="A1:D85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1748,6 +1748,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>0.0007970100000000008</v>
+      </c>
+      <c r="C85" t="n">
+        <v>62107.12538111184</v>
+      </c>
+      <c r="D85" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-06-14
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D85"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1764,6 +1764,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>06/14/2026</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>0.0007659199999999963</v>
+      </c>
+      <c r="C86" t="n">
+        <v>64628.15959891403</v>
+      </c>
+      <c r="D86" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-06-21
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D86"/>
+  <dimension ref="A1:D87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1780,6 +1780,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>06/21/2026</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>0.0007664900000000086</v>
+      </c>
+      <c r="C87" t="n">
+        <v>64580.09889235273</v>
+      </c>
+      <c r="D87" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-06-28
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D87"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1796,6 +1796,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>06/28/2026</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>0.0008233199999999954</v>
+      </c>
+      <c r="C88" t="n">
+        <v>60122.43113248831</v>
+      </c>
+      <c r="D88" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-07-05
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D88"/>
+  <dimension ref="A1:D89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1812,6 +1812,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>0.0007858199999999996</v>
+      </c>
+      <c r="C89" t="n">
+        <v>62991.52477666645</v>
+      </c>
+      <c r="D89" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-07-12
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D89"/>
+  <dimension ref="A1:D90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1828,6 +1828,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>07/12/2026</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>0.001155690000000001</v>
+      </c>
+      <c r="C90" t="n">
+        <v>64247.33276224588</v>
+      </c>
+      <c r="D90" t="n">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-07-19
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D90"/>
+  <dimension ref="A1:D91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1844,6 +1844,22 @@
         <v>75</v>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>07/19/2026</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>0.001143140000000001</v>
+      </c>
+      <c r="C91" t="n">
+        <v>64952.6742131322</v>
+      </c>
+      <c r="D91" t="n">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-07-26
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D91"/>
+  <dimension ref="A1:D92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1860,6 +1860,22 @@
         <v>75</v>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>07/26/2026</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>0.001147389999999998</v>
+      </c>
+      <c r="C92" t="n">
+        <v>64712.08569013162</v>
+      </c>
+      <c r="D92" t="n">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-08-02
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D92"/>
+  <dimension ref="A1:D93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1876,6 +1876,22 @@
         <v>75</v>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>08/02/2026</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>0.001166050000000002</v>
+      </c>
+      <c r="C93" t="n">
+        <v>63676.51472921392</v>
+      </c>
+      <c r="D93" t="n">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-08-09
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D93"/>
+  <dimension ref="A1:D94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1892,6 +1892,22 @@
         <v>75</v>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>0.001141469999999999</v>
+      </c>
+      <c r="C94" t="n">
+        <v>65047.70164787519</v>
+      </c>
+      <c r="D94" t="n">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-08-16
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D94"/>
+  <dimension ref="A1:D95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1908,6 +1908,22 @@
         <v>75</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>08/16/2026</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>0.001172739999999999</v>
+      </c>
+      <c r="C95" t="n">
+        <v>63313.26636765191</v>
+      </c>
+      <c r="D95" t="n">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-08-23
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D95"/>
+  <dimension ref="A1:D96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1924,6 +1924,22 @@
         <v>75</v>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>08/23/2026</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>0.0009700899999999998</v>
+      </c>
+      <c r="C96" t="n">
+        <v>76539.2901689534</v>
+      </c>
+      <c r="D96" t="n">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-08-30
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D96"/>
+  <dimension ref="A1:D97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1940,6 +1940,22 @@
         <v>75</v>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>08/30/2026</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>0.0009456200000000012</v>
+      </c>
+      <c r="C97" t="n">
+        <v>78519.91286140301</v>
+      </c>
+      <c r="D97" t="n">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-09-06
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1956,6 +1956,22 @@
         <v>75</v>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>09/06/2026</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>0.0009226099999999973</v>
+      </c>
+      <c r="C98" t="n">
+        <v>80478.20856049708</v>
+      </c>
+      <c r="D98" t="n">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update bitcoin_buys.xlsx after running on 2026-09-13
</commit_message>
<xml_diff>
--- a/data/bitcoin_buys.xlsx
+++ b/data/bitcoin_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D98"/>
+  <dimension ref="A1:D99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1972,6 +1972,22 @@
         <v>75</v>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>09/13/2026</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>0.0009561300000000064</v>
+      </c>
+      <c r="C99" t="n">
+        <v>77656.80399108856</v>
+      </c>
+      <c r="D99" t="n">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>